<commit_message>
Cambios en importacion excel
</commit_message>
<xml_diff>
--- a/TomaInventarioWEB/Plantillas/Plantilla_Detalle.xlsx
+++ b/TomaInventarioWEB/Plantillas/Plantilla_Detalle.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Carlos Figueroa\Proyectos 2024\Toma Inventarios\Fuente\TomaInventario\TomaInventarioWEB_IQFARMA\TomaInventarioWEB\Plantillas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\User\Desktop\Documentos\TomaDeInventario - Web\TomaInventario-GitHub\TomaInventarioWEB\Plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7568406A-93E6-4139-87FE-E9B56BF87D24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E43977DE-0DB9-4502-8B8C-E464DAA591B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27750" yWindow="1110" windowWidth="20880" windowHeight="11835" tabRatio="983" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30120" yWindow="1050" windowWidth="25425" windowHeight="14160" tabRatio="983" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="18" r:id="rId1"/>
@@ -22,23 +22,23 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
-    <t>COD_UBICACION</t>
+    <t>CÓDIGO DE UBICACIÓN</t>
   </si>
   <si>
-    <t>COD_PRODUCTO</t>
+    <t>CÓDIGO DE PRODUCTO</t>
   </si>
   <si>
-    <t>LOTE_PRODUCTO</t>
+    <t>LOTE DE PRODUCTO</t>
   </si>
   <si>
-    <t>STOCK_ACTUAL</t>
+    <t>STOCK ACTUAL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -53,8 +53,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -64,6 +71,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -93,14 +106,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -408,30 +422,30 @@
   <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:4" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
     </row>
   </sheetData>
   <dataConsolidate/>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThan" showInputMessage="1" showErrorMessage="1" sqref="D1:D1048576" xr:uid="{80D628C6-A0B9-4059-AF4C-4BF28B3603A7}">
+    <dataValidation type="decimal" operator="greaterThan" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576" xr:uid="{80D628C6-A0B9-4059-AF4C-4BF28B3603A7}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>